<commit_message>
add more scripts to mongo's 2-Invoice-Recon. These sctipts calculate the report independently under misc_reports
</commit_message>
<xml_diff>
--- a/eastel-report-scripts/reports-pipelines/report-generation-mongo/2-Invoice-Recon/2-Invoice-Recon-actual-queries-used-output-file.xlsx
+++ b/eastel-report-scripts/reports-pipelines/report-generation-mongo/2-Invoice-Recon/2-Invoice-Recon-actual-queries-used-output-file.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,6 +433,199 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Q014</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>D:\DB_repos\eastel-reports\eastel-report-scripts\reports-pipelines\report-generation-mongo\2-Invoice-Recon\queries\14.js</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 14: Premium and special numbers.
+Output columns:
+- service_type
+- charge_type
+- call_type
+- no_of_calls
+- mou
+*/
+db.usage_logs.aggregate([
+  {
+    $match: {
+      usage_start_time: {
+        $gte: ISODate("2026-04-01T00:00:00Z"),
+        $lt: ISODate("2026-05-01T00:00:00Z")
+      },
+      rat_type: "VO",
+      service_type_sub_cd: "MO",
+      roaming_destination_id: 87,
+      act_usage_unit: { $gt: 0 },
+      $or: [
+        { opposite_number: "600380008000" },
+        { opposite_number: "60103" },
+        { opposite_number: "60100" },
+        { opposite_number: "6015454" },
+        { opposite_number: "6015300" },
+        { opposite_number: "6015353" },
+        { opposite_number: "6015404" },
+        { opposite_number: "6015444" },
+        { opposite_number: "6015777" },
+        { opposite_number: "6015555" },
+        { opposite_number: "6015999" },
+        { opposite_number: "6013504" },
+        { opposite_number: "6015511" },
+        { opposite_number: "6015800" },
+        { opposite_number: "6015995" },
+        { opposite_number: { $regex: "^601300" } },
+        { opposite_number: { $regex: "^601700" } },
+        { opposite_number: { $regex: "^601800" } }
+      ]
+    }
+  },
+  {
+    $addFields: {
+      call_type: {
+        $switch: {
+          branches: [
+            { case: { $eq: ["$opposite_number", "600380008000"] }, then: "1 MOCC - 03-8000 8000" },
+            {
+              case: {
+                $and: [
+                  { $regexMatch: { input: { $ifNull: ["$opposite_number", ""] }, regex: "^601300" } },
+                  { $lt: [{ $strLenCP: { $ifNull: ["$opposite_number", ""] } }, 12] }
+                ]
+              },
+              then: "1300 Numbers"
+            },
+            {
+              case: {
+                $and: [
+                  { $regexMatch: { input: { $ifNull: ["$opposite_number", ""] }, regex: "^601700" } },
+                  { $lt: [{ $strLenCP: { $ifNull: ["$opposite_number", ""] } }, 12] }
+                ]
+              },
+              then: "1700 Numbers"
+            },
+            {
+              case: {
+                $and: [
+                  { $regexMatch: { input: { $ifNull: ["$opposite_number", ""] }, regex: "^601800" } },
+                  { $lt: [{ $strLenCP: { $ifNull: ["$opposite_number", ""] } }, 12] }
+                ]
+              },
+              then: "1800 Numbers"
+            },
+            { case: { $eq: ["$opposite_number", "60103"] }, then: "Directory Assistance -Services 103" },
+            { case: { $eq: ["$opposite_number", "60100"] }, then: "Info Services - 100" },
+            { case: { $eq: ["$opposite_number", "6015454"] }, then: "Info Services - 15454" },
+            { case: { $eq: ["$opposite_number", "6015300"] }, then: "Info Services - 15300" },
+            { case: { $eq: ["$opposite_number", "6015353"] }, then: "Info Services - 15353" },
+            { case: { $eq: ["$opposite_number", "6015404"] }, then: "Info Services - 15404" },
+            { case: { $eq: ["$opposite_number", "6015444"] }, then: "Info Services - 15444" },
+            { case: { $eq: ["$opposite_number", "6015777"] }, then: "Info Services - 15777" },
+            { case: { $eq: ["$opposite_number", "6015555"] }, then: "Info Services - 15555" },
+            { case: { $eq: ["$opposite_number", "6015999"] }, then: "Info Services - 15999" },
+            { case: { $eq: ["$opposite_number", "6013504"] }, then: "Info Services - 13504" },
+            { case: { $eq: ["$opposite_number", "6015511"] }, then: "Info Services - 15511" },
+            { case: { $eq: ["$opposite_number", "6015800"] }, then: "Info Services - 15800" },
+            { case: { $eq: ["$opposite_number", "6015995"] }, then: "Info Services - 15995" }
+          ],
+          default: null
+        }
+      }
+    }
+  },
+  {
+    $match: {
+      call_type: { $ne: null }
+    }
+  },
+  {
+    $group: {
+      _id: "$call_type",
+      no_of_calls: { $sum: 1 },
+      mou: {
+        $sum: {
+          $divide: [
+            { $toDouble: { $ifNull: ["$act_usage_unit", 0] } },
+            60
+          ]
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Voice" },
+      charge_type: { $literal: "Premium and Special Numbers" },
+      call_type: "$_id",
+      no_of_calls: 1,
+      mou: 1,
+      sort_order: {
+        $switch: {
+          branches: [
+            { case: { $eq: ["$_id", "1 MOCC - 03-8000 8000"] }, then: 1 },
+            { case: { $eq: ["$_id", "1300 Numbers"] }, then: 2 },
+            { case: { $eq: ["$_id", "1700 Numbers"] }, then: 3 },
+            { case: { $eq: ["$_id", "1800 Numbers"] }, then: 4 },
+            { case: { $eq: ["$_id", "Directory Assistance -Services 103"] }, then: 5 },
+            { case: { $eq: ["$_id", "Info Services - 100"] }, then: 7 },
+            { case: { $eq: ["$_id", "Info Services - 15454"] }, then: 8 },
+            { case: { $eq: ["$_id", "Info Services - 15300"] }, then: 9 },
+            { case: { $eq: ["$_id", "Info Services - 15353"] }, then: 10 },
+            { case: { $eq: ["$_id", "Info Services - 15404"] }, then: 11 },
+            { case: { $eq: ["$_id", "Info Services - 15444"] }, then: 12 },
+            { case: { $eq: ["$_id", "Info Services - 15777"] }, then: 13 },
+            { case: { $eq: ["$_id", "Info Services - 15555"] }, then: 14 },
+            { case: { $eq: ["$_id", "Info Services - 15999"] }, then: 15 },
+            { case: { $eq: ["$_id", "Info Services - 13504"] }, then: 16 },
+            { case: { $eq: ["$_id", "Info Services - 15511"] }, then: 17 },
+            { case: { $eq: ["$_id", "Info Services - 15800"] }, then: 18 },
+            { case: { $eq: ["$_id", "Info Services - 15995"] }, then: 19 }
+          ],
+          default: 999
+        }
+      }
+    }
+  },
+  {
+    $addFields: {
+      mou: { $round: ["$mou", 2] }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: 1,
+      charge_type: 1,
+      call_type: 1,
+      no_of_calls: 1,
+      mou: 1,
+      sort_order: 1
+    }
+  },
+  {
+    $sort: {
+      sort_order: 1
+    }
+  },
+  {
+    $project: {
+      sort_order: 0
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>